<commit_message>
Added minimal enemy logic Bug fix:  - Now MoveRegistry read correctly from the chosen resource Added MoveRegistryTest class Adjusted MoveReaderTest class logic Upgraded Excel Test
</commit_message>
<xml_diff>
--- a/Test.xlsx
+++ b/Test.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29629"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unipa-my.sharepoint.com/personal/giulia_filicicchia_you_unipa_it/Documents/3° anno/1° semestre/Ingegneria e sicurezza del software/Progetto/iss-team2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="468" documentId="8_{29DD951C-528A-4776-8463-3B1196B446A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48C250FB-F1F6-43B9-806E-812507A9EAC9}"/>
+  <xr:revisionPtr revIDLastSave="550" documentId="8_{29DD951C-528A-4776-8463-3B1196B446A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A977854F-7BE8-421F-B5AC-26EDF79AD137}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C5A1575A-BDFF-4E49-8C7D-0AF3FDC18191}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="201">
   <si>
     <t>ID</t>
   </si>
@@ -62,12 +62,12 @@
     <t>Risultato Atteso</t>
   </si>
   <si>
+    <t>Party</t>
+  </si>
+  <si>
     <t>T1</t>
   </si>
   <si>
-    <t>Party</t>
-  </si>
-  <si>
     <t>Party(List&lt;Player&gt;)</t>
   </si>
   <si>
@@ -173,21 +173,6 @@
     <t>Player</t>
   </si>
   <si>
-    <t>testAddXp()</t>
-  </si>
-  <si>
-    <t>Riceve xp</t>
-  </si>
-  <si>
-    <t>xp non negativa</t>
-  </si>
-  <si>
-    <t>addXp(xp)</t>
-  </si>
-  <si>
-    <t>xp si somma a player.xp</t>
-  </si>
-  <si>
     <t>testNotifyFollower()</t>
   </si>
   <si>
@@ -200,7 +185,64 @@
     <t>notifyFollower()</t>
   </si>
   <si>
-    <t>La posizione dei players diventaquella del player che stanno seguendo</t>
+    <t>La posizione dei players diventa quella del player che stanno seguendo</t>
+  </si>
+  <si>
+    <t>StaticSpeedTurn</t>
+  </si>
+  <si>
+    <t>testSortAction()</t>
+  </si>
+  <si>
+    <t>Si svolge un turno di Battaglia</t>
+  </si>
+  <si>
+    <t>sortAction()</t>
+  </si>
+  <si>
+    <t>La lista contenuta in StaticSpeedTurn è ordinata correttamente dal CharacterPG più veloce al meno veloce</t>
+  </si>
+  <si>
+    <t>testGetTurnIterator()</t>
+  </si>
+  <si>
+    <t>getTurnIterator()</t>
+  </si>
+  <si>
+    <t>Il ConcreteTurnIterator itera correttamente all'interno della lista</t>
+  </si>
+  <si>
+    <t>MoveReader</t>
+  </si>
+  <si>
+    <t>testReadMove()</t>
+  </si>
+  <si>
+    <t>Viene riempito il MoveRegistry</t>
+  </si>
+  <si>
+    <t>"/battle/moves.json"</t>
+  </si>
+  <si>
+    <t>readMove(path)</t>
+  </si>
+  <si>
+    <t>Viene restituita una lista contenente tutte le mosse descritte nella risorsa specificata per come specificata nella classe Move</t>
+  </si>
+  <si>
+    <t>MoveRegistry</t>
+  </si>
+  <si>
+    <t>testGetMoveRegistry</t>
+  </si>
+  <si>
+    <t>Viene richiamata una ActionStrategy a partire dal nome della Move</t>
+  </si>
+  <si>
+    <t>getMoveRegistry()</t>
+  </si>
+  <si>
+    <t>MoveRegistry mappa correttamente tutte le Move contenute in "moves.json"</t>
   </si>
   <si>
     <t>Position(x,y)</t>
@@ -606,7 +648,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -654,10 +696,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -994,17 +1039,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35400F29-09C1-4308-BA0B-71DD5C94186E}">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="3" max="3" width="23.6640625" customWidth="1"/>
-    <col min="4" max="4" width="38.5546875" customWidth="1"/>
-    <col min="5" max="5" width="21.33203125" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" customWidth="1"/>
+    <col min="4" max="4" width="38.5703125" customWidth="1"/>
+    <col min="5" max="5" width="21.28515625" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="55.21875" customWidth="1"/>
+    <col min="7" max="7" width="55.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1027,212 +1073,296 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:7" ht="15">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:7" ht="15">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D3" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E3" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="4" spans="1:7" ht="15">
+      <c r="A4" t="s">
         <v>14</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>15</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D4" t="s">
         <v>16</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E4" t="s">
         <v>17</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F4" t="s">
         <v>15</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="5" spans="1:7" ht="15">
+      <c r="A5" t="s">
         <v>19</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
         <v>20</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D5" t="s">
         <v>21</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E5" t="s">
         <v>22</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F5" t="s">
         <v>20</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="6" spans="1:7" ht="15">
+      <c r="A6" t="s">
         <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>29</v>
       </c>
       <c r="C6" t="s">
         <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E6" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s">
         <v>25</v>
       </c>
       <c r="G6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
         <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E7" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F7" t="s">
         <v>25</v>
       </c>
       <c r="G7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    <row r="9" spans="1:7" ht="15">
+      <c r="A9" t="s">
         <v>37</v>
       </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" t="s">
         <v>38</v>
-      </c>
-      <c r="E8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" t="s">
-        <v>42</v>
       </c>
       <c r="E9" t="s">
         <v>39</v>
       </c>
       <c r="F9" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" t="s">
+    <row r="10" spans="1:7" ht="15">
+      <c r="A10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15">
+      <c r="B13" t="s">
         <v>43</v>
       </c>
-      <c r="C12" t="s">
+    </row>
+    <row r="14" spans="1:7" ht="29.25">
+      <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
         <v>44</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D14" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E14" t="s">
         <v>46</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F14" t="s">
         <v>47</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G14" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+    <row r="15" spans="1:7" ht="15"/>
+    <row r="16" spans="1:7" ht="15"/>
+    <row r="17" spans="1:7" ht="15">
+      <c r="B17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="29.25">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" t="s">
+        <v>51</v>
+      </c>
+      <c r="F18" t="s">
+        <v>52</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
         <v>14</v>
       </c>
-      <c r="C13" t="s">
-        <v>49</v>
-      </c>
-      <c r="D13" t="s">
-        <v>50</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="C19" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" t="s">
         <v>51</v>
       </c>
-      <c r="F13" t="s">
-        <v>52</v>
-      </c>
-      <c r="G13" t="s">
-        <v>53</v>
-      </c>
-    </row>
+      <c r="F19" t="s">
+        <v>55</v>
+      </c>
+      <c r="G19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" s="2" customFormat="1" ht="15">
+      <c r="A22"/>
+      <c r="B22" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22"/>
+      <c r="D22"/>
+      <c r="E22"/>
+      <c r="F22"/>
+      <c r="G22"/>
+    </row>
+    <row r="23" spans="1:7" ht="29.25">
+      <c r="A23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" t="s">
+        <v>59</v>
+      </c>
+      <c r="E23" t="s">
+        <v>60</v>
+      </c>
+      <c r="F23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15"/>
+    <row r="25" spans="1:7" ht="15"/>
+    <row r="26" spans="1:7" ht="15">
+      <c r="B26" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="29.25">
+      <c r="A27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15"/>
+    <row r="31" spans="1:7" ht="15"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1242,16 +1372,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2FB2765-FCFC-41A8-8777-28375534F16F}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="2" max="2" width="23.109375" customWidth="1"/>
-    <col min="3" max="3" width="24.88671875" customWidth="1"/>
-    <col min="4" max="4" width="27.6640625" customWidth="1"/>
-    <col min="5" max="5" width="19.44140625" customWidth="1"/>
-    <col min="6" max="6" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" customWidth="1"/>
+    <col min="4" max="4" width="27.7109375" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" customWidth="1"/>
+    <col min="6" max="6" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1271,224 +1401,224 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="F2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="F3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="C4" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="E4" t="s">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="E5" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="F5" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="D6" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="E6" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="F6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="D7" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="E7" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="F7" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="C8" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="D8" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="E8" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="F8" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="C9" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="D9" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="E9" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="F9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="C10" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="D10" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="E10" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="F10" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="C11" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="D11" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="E11" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="F11" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="B12" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="C12" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="D12" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="E12" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="F12" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1500,16 +1630,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3C4191E-2A78-4707-924F-805E6AC0DF21}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="29.88671875" customWidth="1"/>
-    <col min="4" max="4" width="43.6640625" customWidth="1"/>
-    <col min="5" max="5" width="36.33203125" customWidth="1"/>
-    <col min="6" max="6" width="38.88671875" customWidth="1"/>
+    <col min="3" max="3" width="29.85546875" customWidth="1"/>
+    <col min="4" max="4" width="43.7109375" customWidth="1"/>
+    <col min="5" max="5" width="36.28515625" customWidth="1"/>
+    <col min="6" max="6" width="38.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1529,164 +1659,164 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="C2" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="D2" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="E2" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="F2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="C3" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="D3" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="E3" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="F3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="C4" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="D4" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="E4" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="F4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="C5" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="D5" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="E5" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="F5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C6" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="D6" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="E6" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="F6" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="F7" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="C8" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="D8" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="E8" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="F8" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="C9" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="D9" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="E9" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="F9" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -1697,17 +1827,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC088249-D306-499A-B716-BF709674AF2A}">
   <dimension ref="A1:F16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="2" max="2" width="17.44140625" customWidth="1"/>
-    <col min="3" max="3" width="22.33203125" customWidth="1"/>
-    <col min="4" max="4" width="33.5546875" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" customWidth="1"/>
+    <col min="4" max="4" width="33.5703125" customWidth="1"/>
     <col min="5" max="5" width="32" customWidth="1"/>
     <col min="6" max="6" width="34" customWidth="1"/>
-    <col min="7" max="7" width="19.6640625" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1727,304 +1857,304 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="C2" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="D2" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="E2" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="F2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C3" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="D3" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="E3" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="F3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="C4" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="D4" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="E4" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="F4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="C5" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="D5" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="E5" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="F5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="C6" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="D6" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="E6" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="F6" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="C7" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="D7" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="E7" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="F7" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="C8" t="s">
+        <v>172</v>
+      </c>
+      <c r="D8" t="s">
+        <v>173</v>
+      </c>
+      <c r="E8" t="s">
         <v>158</v>
       </c>
-      <c r="D8" t="s">
-        <v>159</v>
-      </c>
-      <c r="E8" t="s">
-        <v>144</v>
-      </c>
       <c r="F8" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="C9" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="D9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E9" t="s">
+        <v>158</v>
+      </c>
+      <c r="F9" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>99</v>
+      </c>
+      <c r="B10" t="s">
         <v>162</v>
       </c>
-      <c r="E9" t="s">
-        <v>144</v>
-      </c>
-      <c r="F9" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>85</v>
-      </c>
-      <c r="B10" t="s">
-        <v>148</v>
-      </c>
       <c r="C10" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="D10" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="E10" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="F10" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="B11" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="C11" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="D11" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="E11" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="F11" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="B12" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="C12" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="D12" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="E12" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="F12" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="B13" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="C13" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="D13" t="s">
+        <v>188</v>
+      </c>
+      <c r="E13" t="s">
+        <v>158</v>
+      </c>
+      <c r="F13" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>190</v>
+      </c>
+      <c r="B14" t="s">
+        <v>162</v>
+      </c>
+      <c r="C14" t="s">
+        <v>191</v>
+      </c>
+      <c r="D14" t="s">
+        <v>192</v>
+      </c>
+      <c r="E14" t="s">
+        <v>158</v>
+      </c>
+      <c r="F14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>194</v>
+      </c>
+      <c r="B15" t="s">
+        <v>162</v>
+      </c>
+      <c r="C15" t="s">
+        <v>195</v>
+      </c>
+      <c r="D15" t="s">
+        <v>196</v>
+      </c>
+      <c r="E15" t="s">
+        <v>158</v>
+      </c>
+      <c r="F15" t="s">
         <v>174</v>
       </c>
-      <c r="E13" t="s">
-        <v>144</v>
-      </c>
-      <c r="F13" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>176</v>
-      </c>
-      <c r="B14" t="s">
-        <v>148</v>
-      </c>
-      <c r="C14" t="s">
-        <v>177</v>
-      </c>
-      <c r="D14" t="s">
-        <v>178</v>
-      </c>
-      <c r="E14" t="s">
-        <v>144</v>
-      </c>
-      <c r="F14" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>180</v>
-      </c>
-      <c r="B15" t="s">
-        <v>148</v>
-      </c>
-      <c r="C15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D15" t="s">
-        <v>182</v>
-      </c>
-      <c r="E15" t="s">
-        <v>144</v>
-      </c>
-      <c r="F15" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>183</v>
+        <v>197</v>
       </c>
       <c r="B16" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="C16" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
       <c r="D16" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
       <c r="E16" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="F16" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tests for exploration controller
</commit_message>
<xml_diff>
--- a/Test.xlsx
+++ b/Test.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unipa-my.sharepoint.com/personal/giulia_filicicchia_you_unipa_it/Documents/3° anno/1° semestre/Ingegneria e sicurezza del software/Progetto/iss-team2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unipa-my.sharepoint.com/personal/samuelemaria_morreale_you_unipa_it/Documents/3anno/appunti e dispense/ingegneria del software/progetto/iss-team2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="835" documentId="8_{29DD951C-528A-4776-8463-3B1196B446A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{477640BE-F15C-4AF8-B672-B67D4FCE6A38}"/>
+  <xr:revisionPtr revIDLastSave="851" documentId="8_{29DD951C-528A-4776-8463-3B1196B446A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A88A6947-EF28-4AB7-A3FA-EC3DFFC8898C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C5A1575A-BDFF-4E49-8C7D-0AF3FDC18191}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="274">
   <si>
     <t>ID</t>
   </si>
@@ -386,9 +386,6 @@
     <t>Creazione controller</t>
   </si>
   <si>
-    <t>Party valido, Scene(800x600),speed=32</t>
-  </si>
-  <si>
     <t>new MovementController</t>
   </si>
   <si>
@@ -401,9 +398,6 @@
     <t>Calcolo limiti posizione</t>
   </si>
   <si>
-    <t>Scene(800x600), speed=32</t>
-  </si>
-  <si>
     <t>posLimit coerente con dimensioni scene</t>
   </si>
   <si>
@@ -440,12 +434,6 @@
     <t>Posizione invariata</t>
   </si>
   <si>
-    <t>Direzione opposta</t>
-  </si>
-  <si>
-    <t>prev=W, key=S</t>
-  </si>
-  <si>
     <t>Nessun movimento</t>
   </si>
   <si>
@@ -509,12 +497,6 @@
     <t>T14</t>
   </si>
   <si>
-    <t>speed=0</t>
-  </si>
-  <si>
-    <t>key=0</t>
-  </si>
-  <si>
     <t>T15</t>
   </si>
   <si>
@@ -689,9 +671,6 @@
     <t>Enemy nella stessa posizione del main player</t>
   </si>
   <si>
-    <t>battleStarted=true</t>
-  </si>
-  <si>
     <t>Battle iniziato</t>
   </si>
   <si>
@@ -722,9 +701,6 @@
     <t>Player spostato</t>
   </si>
   <si>
-    <t>T19</t>
-  </si>
-  <si>
     <t>testLearnMove()</t>
   </si>
   <si>
@@ -873,6 +849,15 @@
   </si>
   <si>
     <t>file autosave.json non presente</t>
+  </si>
+  <si>
+    <t>Party valido, Scene(800x600)</t>
+  </si>
+  <si>
+    <t>Scene(800x600)</t>
+  </si>
+  <si>
+    <t>handleBattle chiamato</t>
   </si>
 </sst>
 </file>
@@ -974,10 +959,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1297,7 +1278,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35400F29-09C1-4308-BA0B-71DD5C94186E}">
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="20.44140625" customWidth="1"/>
@@ -1535,7 +1516,7 @@
         <v>101</v>
       </c>
       <c r="F15" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="G15" t="s">
         <v>102</v>
@@ -1566,7 +1547,7 @@
         <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="D17" t="s">
         <v>112</v>
@@ -1575,7 +1556,7 @@
         <v>113</v>
       </c>
       <c r="F17" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="G17" t="s">
         <v>114</v>
@@ -1606,19 +1587,19 @@
         <v>33</v>
       </c>
       <c r="C19" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="D19" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="E19" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="F19" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="G19" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -1634,7 +1615,7 @@
         <v>50</v>
       </c>
       <c r="D21" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="F21" t="s">
         <v>51</v>
@@ -1646,7 +1627,7 @@
     <row r="23" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23"/>
       <c r="B23" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="C23"/>
       <c r="D23"/>
@@ -1659,16 +1640,16 @@
         <v>8</v>
       </c>
       <c r="C24" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D24" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="E24" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="G24" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -1676,12 +1657,12 @@
         <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -1906,7 +1887,7 @@
     </row>
     <row r="40" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B40" s="5" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
@@ -1914,19 +1895,19 @@
         <v>8</v>
       </c>
       <c r="C41" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D41" t="s">
         <v>115</v>
       </c>
       <c r="E41" t="s">
+        <v>271</v>
+      </c>
+      <c r="F41" t="s">
         <v>116</v>
       </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
         <v>117</v>
-      </c>
-      <c r="G41" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
@@ -1934,19 +1915,19 @@
         <v>14</v>
       </c>
       <c r="C42" t="s">
+        <v>118</v>
+      </c>
+      <c r="D42" t="s">
         <v>119</v>
       </c>
-      <c r="D42" t="s">
-        <v>120</v>
-      </c>
       <c r="E42" t="s">
-        <v>121</v>
+        <v>272</v>
       </c>
       <c r="F42" t="s">
         <v>115</v>
       </c>
       <c r="G42" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
@@ -1954,19 +1935,19 @@
         <v>19</v>
       </c>
       <c r="C43" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D43" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="E43" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="F43" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="G43" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
@@ -1974,19 +1955,19 @@
         <v>24</v>
       </c>
       <c r="C44" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D44" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="E44" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="F44" t="s">
-        <v>217</v>
+        <v>273</v>
       </c>
       <c r="G44" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
@@ -1994,19 +1975,19 @@
         <v>29</v>
       </c>
       <c r="C45" t="s">
+        <v>122</v>
+      </c>
+      <c r="D45" t="s">
+        <v>123</v>
+      </c>
+      <c r="E45" t="s">
         <v>124</v>
       </c>
-      <c r="D45" t="s">
+      <c r="F45" t="s">
+        <v>121</v>
+      </c>
+      <c r="G45" t="s">
         <v>125</v>
-      </c>
-      <c r="E45" t="s">
-        <v>126</v>
-      </c>
-      <c r="F45" t="s">
-        <v>123</v>
-      </c>
-      <c r="G45" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
@@ -2014,19 +1995,19 @@
         <v>33</v>
       </c>
       <c r="C46" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D46" t="s">
+        <v>126</v>
+      </c>
+      <c r="E46" t="s">
+        <v>127</v>
+      </c>
+      <c r="F46" t="s">
+        <v>121</v>
+      </c>
+      <c r="G46" t="s">
         <v>128</v>
-      </c>
-      <c r="E46" t="s">
-        <v>129</v>
-      </c>
-      <c r="F46" t="s">
-        <v>123</v>
-      </c>
-      <c r="G46" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
@@ -2034,99 +2015,99 @@
         <v>37</v>
       </c>
       <c r="C47" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D47" t="s">
+        <v>129</v>
+      </c>
+      <c r="E47" t="s">
+        <v>130</v>
+      </c>
+      <c r="F47" t="s">
+        <v>121</v>
+      </c>
+      <c r="G47" t="s">
         <v>131</v>
-      </c>
-      <c r="E47" t="s">
-        <v>132</v>
-      </c>
-      <c r="F47" t="s">
-        <v>123</v>
-      </c>
-      <c r="G47" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>41</v>
+        <v>84</v>
       </c>
       <c r="C48" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D48" t="s">
+        <v>133</v>
+      </c>
+      <c r="E48" t="s">
         <v>134</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
+        <v>121</v>
+      </c>
+      <c r="G48" t="s">
         <v>135</v>
-      </c>
-      <c r="F48" t="s">
-        <v>123</v>
-      </c>
-      <c r="G48" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C49" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D49" t="s">
+        <v>136</v>
+      </c>
+      <c r="E49" t="s">
         <v>137</v>
       </c>
-      <c r="E49" t="s">
-        <v>138</v>
-      </c>
       <c r="F49" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G49" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C50" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D50" t="s">
+        <v>138</v>
+      </c>
+      <c r="E50" t="s">
+        <v>139</v>
+      </c>
+      <c r="F50" t="s">
+        <v>121</v>
+      </c>
+      <c r="G50" t="s">
         <v>140</v>
-      </c>
-      <c r="E50" t="s">
-        <v>141</v>
-      </c>
-      <c r="F50" t="s">
-        <v>123</v>
-      </c>
-      <c r="G50" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>94</v>
+        <v>144</v>
       </c>
       <c r="C51" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D51" t="s">
+        <v>141</v>
+      </c>
+      <c r="E51" t="s">
         <v>142</v>
       </c>
-      <c r="E51" t="s">
+      <c r="F51" t="s">
+        <v>121</v>
+      </c>
+      <c r="G51" t="s">
         <v>143</v>
-      </c>
-      <c r="F51" t="s">
-        <v>123</v>
-      </c>
-      <c r="G51" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
@@ -2134,7 +2115,7 @@
         <v>148</v>
       </c>
       <c r="C52" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D52" t="s">
         <v>145</v>
@@ -2143,7 +2124,7 @@
         <v>146</v>
       </c>
       <c r="F52" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G52" t="s">
         <v>147</v>
@@ -2154,7 +2135,7 @@
         <v>152</v>
       </c>
       <c r="C53" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D53" t="s">
         <v>149</v>
@@ -2163,7 +2144,7 @@
         <v>150</v>
       </c>
       <c r="F53" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G53" t="s">
         <v>151</v>
@@ -2171,42 +2152,42 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
+        <v>153</v>
+      </c>
+      <c r="C54" t="s">
+        <v>118</v>
+      </c>
+      <c r="D54" t="s">
+        <v>154</v>
+      </c>
+      <c r="E54" t="s">
+        <v>155</v>
+      </c>
+      <c r="F54" t="s">
+        <v>116</v>
+      </c>
+      <c r="G54" t="s">
         <v>156</v>
-      </c>
-      <c r="C54" t="s">
-        <v>124</v>
-      </c>
-      <c r="D54" t="s">
-        <v>153</v>
-      </c>
-      <c r="E54" t="s">
-        <v>154</v>
-      </c>
-      <c r="F54" t="s">
-        <v>123</v>
-      </c>
-      <c r="G54" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>159</v>
+        <v>197</v>
       </c>
       <c r="C55" t="s">
-        <v>124</v>
+        <v>198</v>
       </c>
       <c r="D55" t="s">
-        <v>157</v>
+        <v>199</v>
       </c>
       <c r="E55" t="s">
-        <v>158</v>
+        <v>200</v>
       </c>
       <c r="F55" t="s">
-        <v>123</v>
+        <v>201</v>
       </c>
       <c r="G55" t="s">
-        <v>136</v>
+        <v>202</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
@@ -2214,206 +2195,206 @@
         <v>203</v>
       </c>
       <c r="C56" t="s">
-        <v>119</v>
+        <v>204</v>
       </c>
       <c r="D56" t="s">
-        <v>160</v>
+        <v>205</v>
       </c>
       <c r="E56" t="s">
-        <v>161</v>
+        <v>206</v>
       </c>
       <c r="F56" t="s">
-        <v>117</v>
+        <v>208</v>
       </c>
       <c r="G56" t="s">
-        <v>162</v>
+        <v>207</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C57" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="D57" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="E57" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="F57" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="G57" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>219</v>
-      </c>
-      <c r="C58" t="s">
-        <v>210</v>
-      </c>
-      <c r="D58" t="s">
-        <v>211</v>
-      </c>
-      <c r="E58" t="s">
-        <v>212</v>
-      </c>
-      <c r="F58" t="s">
-        <v>214</v>
-      </c>
-      <c r="G58" t="s">
-        <v>213</v>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B58" s="4" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>228</v>
+        <v>8</v>
       </c>
       <c r="C59" t="s">
-        <v>220</v>
+        <v>174</v>
       </c>
       <c r="D59" t="s">
-        <v>221</v>
+        <v>177</v>
       </c>
       <c r="E59" t="s">
-        <v>222</v>
+        <v>182</v>
       </c>
       <c r="F59" t="s">
-        <v>223</v>
+        <v>192</v>
       </c>
       <c r="G59" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="4" t="s">
-        <v>179</v>
+        <v>187</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>14</v>
+      </c>
+      <c r="C60" t="s">
+        <v>175</v>
+      </c>
+      <c r="D60" t="s">
+        <v>178</v>
+      </c>
+      <c r="E60" t="s">
+        <v>183</v>
+      </c>
+      <c r="F60" t="s">
+        <v>193</v>
+      </c>
+      <c r="G60" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C61" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D61" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="E61" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="F61" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="G61" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C62" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="D62" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="E62" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="F62" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="G62" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C63" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D63" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="E63" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="F63" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="G63" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
-        <v>24</v>
-      </c>
-      <c r="C64" t="s">
-        <v>182</v>
-      </c>
-      <c r="D64" t="s">
-        <v>186</v>
-      </c>
-      <c r="E64" t="s">
         <v>191</v>
       </c>
-      <c r="F64" t="s">
-        <v>201</v>
-      </c>
-      <c r="G64" t="s">
-        <v>196</v>
+    </row>
+    <row r="64" spans="1:7" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B64" s="6" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="C65" t="s">
-        <v>182</v>
+        <v>222</v>
       </c>
       <c r="D65" t="s">
-        <v>187</v>
+        <v>225</v>
       </c>
       <c r="E65" t="s">
-        <v>192</v>
+        <v>234</v>
       </c>
       <c r="F65" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="G65" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B66" s="6" t="s">
-        <v>231</v>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>14</v>
+      </c>
+      <c r="C66" t="s">
+        <v>222</v>
+      </c>
+      <c r="D66" t="s">
+        <v>229</v>
+      </c>
+      <c r="E66" t="s">
+        <v>234</v>
+      </c>
+      <c r="F66" t="s">
+        <v>227</v>
+      </c>
+      <c r="G66" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C67" t="s">
+        <v>228</v>
+      </c>
+      <c r="D67" t="s">
         <v>230</v>
       </c>
-      <c r="D67" t="s">
-        <v>233</v>
-      </c>
       <c r="E67" t="s">
-        <v>242</v>
+        <v>270</v>
       </c>
       <c r="F67" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G67" t="s">
         <v>93</v>
@@ -2421,19 +2402,19 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C68" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D68" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="E68" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="F68" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="G68" t="s">
         <v>89</v>
@@ -2441,30 +2422,30 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C69" t="s">
+        <v>235</v>
+      </c>
+      <c r="D69" t="s">
         <v>236</v>
       </c>
-      <c r="D69" t="s">
+      <c r="E69" t="s">
+        <v>237</v>
+      </c>
+      <c r="F69" t="s">
         <v>238</v>
       </c>
-      <c r="E69" t="s">
-        <v>278</v>
-      </c>
-      <c r="F69" t="s">
+      <c r="G69" t="s">
         <v>239</v>
-      </c>
-      <c r="G69" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C70" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D70" t="s">
         <v>240</v>
@@ -2473,64 +2454,61 @@
         <v>241</v>
       </c>
       <c r="F70" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="G70" t="s">
-        <v>89</v>
+        <v>243</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C71" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D71" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E71" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F71" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G71" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="C72" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="D72" t="s">
-        <v>248</v>
-      </c>
-      <c r="E72" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F72" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G72" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>37</v>
+        <v>84</v>
       </c>
       <c r="C73" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D73" t="s">
         <v>253</v>
       </c>
       <c r="E73" t="s">
-        <v>254</v>
+        <v>224</v>
       </c>
       <c r="F73" t="s">
         <v>255</v>
@@ -2541,7 +2519,7 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>41</v>
+        <v>90</v>
       </c>
       <c r="C74" t="s">
         <v>257</v>
@@ -2549,108 +2527,71 @@
       <c r="D74" t="s">
         <v>258</v>
       </c>
+      <c r="E74" t="s">
+        <v>254</v>
+      </c>
       <c r="F74" t="s">
         <v>259</v>
       </c>
       <c r="G74" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="C75" t="s">
         <v>257</v>
       </c>
       <c r="D75" t="s">
+        <v>260</v>
+      </c>
+      <c r="F75" t="s">
+        <v>259</v>
+      </c>
+      <c r="G75" t="s">
         <v>261</v>
-      </c>
-      <c r="E75" t="s">
-        <v>232</v>
-      </c>
-      <c r="F75" t="s">
-        <v>263</v>
-      </c>
-      <c r="G75" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>90</v>
+        <v>144</v>
       </c>
       <c r="C76" t="s">
+        <v>262</v>
+      </c>
+      <c r="D76" t="s">
+        <v>263</v>
+      </c>
+      <c r="E76" t="s">
+        <v>264</v>
+      </c>
+      <c r="F76" t="s">
         <v>265</v>
       </c>
-      <c r="D76" t="s">
+      <c r="G76" t="s">
         <v>266</v>
-      </c>
-      <c r="E76" t="s">
-        <v>262</v>
-      </c>
-      <c r="F76" t="s">
-        <v>267</v>
-      </c>
-      <c r="G76" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>94</v>
+        <v>148</v>
       </c>
       <c r="C77" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D77" t="s">
+        <v>267</v>
+      </c>
+      <c r="E77" t="s">
+        <v>224</v>
+      </c>
+      <c r="F77" t="s">
         <v>268</v>
-      </c>
-      <c r="F77" t="s">
-        <v>267</v>
       </c>
       <c r="G77" t="s">
         <v>269</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
-        <v>148</v>
-      </c>
-      <c r="C78" t="s">
-        <v>270</v>
-      </c>
-      <c r="D78" t="s">
-        <v>271</v>
-      </c>
-      <c r="E78" t="s">
-        <v>272</v>
-      </c>
-      <c r="F78" t="s">
-        <v>273</v>
-      </c>
-      <c r="G78" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>152</v>
-      </c>
-      <c r="C79" t="s">
-        <v>270</v>
-      </c>
-      <c r="D79" t="s">
-        <v>275</v>
-      </c>
-      <c r="E79" t="s">
-        <v>232</v>
-      </c>
-      <c r="F79" t="s">
-        <v>276</v>
-      </c>
-      <c r="G79" t="s">
-        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added tests for gameController
</commit_message>
<xml_diff>
--- a/Test.xlsx
+++ b/Test.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unipa-my.sharepoint.com/personal/giulia_filicicchia_you_unipa_it/Documents/3° anno/1° semestre/Ingegneria e sicurezza del software/Progetto/iss-team2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unipa-my.sharepoint.com/personal/samuelemaria_morreale_you_unipa_it/Documents/3anno/appunti e dispense/ingegneria del software/progetto/iss-team2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="935" documentId="8_{29DD951C-528A-4776-8463-3B1196B446A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB1839C4-6CB9-4F87-828E-36EFB9A86F3D}"/>
+  <xr:revisionPtr revIDLastSave="997" documentId="8_{29DD951C-528A-4776-8463-3B1196B446A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0D8AF0B-DDF7-479F-B615-44CBE886CDA5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C5A1575A-BDFF-4E49-8C7D-0AF3FDC18191}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="356">
   <si>
     <t>ID</t>
   </si>
@@ -1038,6 +1038,72 @@
   </si>
   <si>
     <t>reward.assiXP chiamato</t>
+  </si>
+  <si>
+    <t>GameController</t>
+  </si>
+  <si>
+    <t>onNewGameConfirmed</t>
+  </si>
+  <si>
+    <t>Creazione di un GameState valido</t>
+  </si>
+  <si>
+    <t>Creazione GameController</t>
+  </si>
+  <si>
+    <t>NewGame</t>
+  </si>
+  <si>
+    <t>new GameController(game)</t>
+  </si>
+  <si>
+    <t>GameController creato senza eccezioni e con attributi corretti</t>
+  </si>
+  <si>
+    <t>GameState.GameStateBuilder.build()</t>
+  </si>
+  <si>
+    <t>GameState creato correttamente</t>
+  </si>
+  <si>
+    <t>players=2, autoSave=false</t>
+  </si>
+  <si>
+    <t>onCharacterSelected</t>
+  </si>
+  <si>
+    <t>Aggiunta di character al GameState</t>
+  </si>
+  <si>
+    <t>Job.ARCHER</t>
+  </si>
+  <si>
+    <t>GameState.selectCharacter()</t>
+  </si>
+  <si>
+    <t>Character aggiunto al party</t>
+  </si>
+  <si>
+    <t>Non aggiunta di character al GameState se party pieno</t>
+  </si>
+  <si>
+    <t>Job.WARRIOR</t>
+  </si>
+  <si>
+    <t>selectCharacter non aggiunge membri al party</t>
+  </si>
+  <si>
+    <t>startExploration</t>
+  </si>
+  <si>
+    <t>Creazione di enemy, party e NPC nel GameState prima di esplorare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GameState.createEnemy, GameState.createParty, GameState.createNpc </t>
+  </si>
+  <si>
+    <t>GameState contiene party, nemici e npc</t>
   </si>
 </sst>
 </file>
@@ -1462,15 +1528,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35400F29-09C1-4308-BA0B-71DD5C94186E}">
-  <dimension ref="A1:G96"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="24.5546875" customWidth="1"/>
-    <col min="3" max="3" width="49.6640625" customWidth="1"/>
-    <col min="4" max="4" width="82.5546875" customWidth="1"/>
-    <col min="5" max="5" width="47.21875" customWidth="1"/>
-    <col min="6" max="6" width="43.44140625" customWidth="1"/>
-    <col min="7" max="7" width="55.33203125" customWidth="1"/>
+    <col min="1" max="1" width="3.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="57.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="64.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="70.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -3109,6 +3176,137 @@
       </c>
       <c r="G96" t="s">
         <v>333</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A98" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G98" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A99" s="6"/>
+      <c r="B99" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="C99" s="6"/>
+      <c r="D99" s="6"/>
+      <c r="E99" s="6"/>
+      <c r="F99" s="6"/>
+      <c r="G99" s="6"/>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>8</v>
+      </c>
+      <c r="C100" t="s">
+        <v>334</v>
+      </c>
+      <c r="D100" t="s">
+        <v>337</v>
+      </c>
+      <c r="E100" t="s">
+        <v>338</v>
+      </c>
+      <c r="F100" t="s">
+        <v>339</v>
+      </c>
+      <c r="G100" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>14</v>
+      </c>
+      <c r="C101" t="s">
+        <v>335</v>
+      </c>
+      <c r="D101" t="s">
+        <v>336</v>
+      </c>
+      <c r="E101" t="s">
+        <v>343</v>
+      </c>
+      <c r="F101" t="s">
+        <v>341</v>
+      </c>
+      <c r="G101" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>19</v>
+      </c>
+      <c r="C102" t="s">
+        <v>344</v>
+      </c>
+      <c r="D102" t="s">
+        <v>345</v>
+      </c>
+      <c r="E102" t="s">
+        <v>346</v>
+      </c>
+      <c r="F102" t="s">
+        <v>347</v>
+      </c>
+      <c r="G102" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>24</v>
+      </c>
+      <c r="C103" t="s">
+        <v>344</v>
+      </c>
+      <c r="D103" t="s">
+        <v>349</v>
+      </c>
+      <c r="E103" t="s">
+        <v>350</v>
+      </c>
+      <c r="F103" t="s">
+        <v>347</v>
+      </c>
+      <c r="G103" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>29</v>
+      </c>
+      <c r="C104" t="s">
+        <v>352</v>
+      </c>
+      <c r="D104" t="s">
+        <v>353</v>
+      </c>
+      <c r="F104" t="s">
+        <v>354</v>
+      </c>
+      <c r="G104" t="s">
+        <v>355</v>
       </c>
     </row>
   </sheetData>

</xml_diff>